<commit_message>
Award: limit qualifying dates to current program year; backfill Jul-Oct 2026
</commit_message>
<xml_diff>
--- a/docs/exports/area/Division_A_Area_01.xlsx
+++ b/docs/exports/area/Division_A_Area_01.xlsx
@@ -514,14 +514,14 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 04 Jul 2026, 13:24  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:25  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Area 01 — Level Totals (Division Rank #2 of 4)</t>
+          <t>Area 01 — Level Totals (Division Rank #1 of 4)</t>
         </is>
       </c>
     </row>
@@ -554,19 +554,19 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>57</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -607,7 +607,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 04 Jul 2026, 13:24  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:25  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -647,19 +647,19 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -710,7 +710,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 04 Jul 2026, 13:24  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:25  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -769,14 +769,14 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>The Colombo Toastmasters Club</t>
+          <t>Commercial Bank Toastmasters Club</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>2</v>
@@ -785,10 +785,10 @@
         <v>2</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>72</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8">
@@ -797,26 +797,26 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Commercial Bank Toastmasters Club</t>
+          <t>Lions Toastmasters Club</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>2</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9">
@@ -825,26 +825,26 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Lions Toastmasters Club</t>
+          <t>CEB Toastmasters Club</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10">
@@ -853,26 +853,26 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>CEB Toastmasters Club</t>
+          <t>The Colombo Toastmasters Club</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="8" t="n">
-        <v>8</v>
-      </c>
       <c r="H10" s="8" t="n">
-        <v>20</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11">
@@ -885,7 +885,7 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" s="6" t="n">
         <v>0</v>
@@ -897,10 +897,10 @@
         <v>0</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -939,7 +939,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 04 Jul 2026, 13:24  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:25  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -987,10 +987,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
   </cols>
@@ -1012,7 +1012,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-06-30  |  Report generated 04 Jul 2026, 13:24  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:25  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -1043,41 +1043,11 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Commercial Bank Toastmasters Club</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Lions Toastmasters Club</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C8" s="8" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>The Colombo Toastmasters Club</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>2</v>
-      </c>
+          <t>No clubs yet</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Read 2026-27 Level 2 column names; stop on missing columns
</commit_message>
<xml_diff>
--- a/docs/exports/area/Division_A_Area_01.xlsx
+++ b/docs/exports/area/Division_A_Area_01.xlsx
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:25  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:31  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -557,7 +557,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>4</v>
@@ -566,7 +566,7 @@
         <v>4</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -607,7 +607,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:25  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:31  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -647,10 +647,10 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>4</v>
@@ -659,7 +659,7 @@
         <v>3</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -710,7 +710,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:25  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:31  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -797,26 +797,26 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Lions Toastmasters Club</t>
+          <t>The Colombo Toastmasters Club</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="F8" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="8" t="n">
-        <v>2</v>
-      </c>
       <c r="G8" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>25</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9">
@@ -825,26 +825,26 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>CEB Toastmasters Club</t>
+          <t>Lions Toastmasters Club</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
@@ -853,26 +853,26 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>The Colombo Toastmasters Club</t>
+          <t>CEB Toastmasters Club</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="8" t="n">
-        <v>0</v>
-      </c>
       <c r="E10" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>0</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>66</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11">
@@ -939,7 +939,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:25  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:31  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:25  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:31  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild reports with Level 2 / OMM label and note
</commit_message>
<xml_diff>
--- a/docs/exports/area/Division_A_Area_01.xlsx
+++ b/docs/exports/area/Division_A_Area_01.xlsx
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:44  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:50  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:44  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:50  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -717,7 +717,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:44  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:50  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:44  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:50  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:44  |  District 82 Toastmasters Pathways Dashboard</t>
+          <t>Data as of 2026-10-20  |  Report generated 21 Oct 2026, 23:50  |  District 82 Toastmasters Pathways Dashboard</t>
         </is>
       </c>
     </row>

</xml_diff>